<commit_message>
Laboratory 05: Structural Breaks Analysis and Model Refinement
</commit_message>
<xml_diff>
--- a/src/netherlands_gva.xlsx
+++ b/src/netherlands_gva.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/danielfaltynowski/Documents/Repositories/netherlands-gva-time-series-analysis/src/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D712139-C96D-AD45-B3AF-41D7A9F9BF9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC739776-944E-2943-AC6B-A47698FECB98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="19400" firstSheet="2" activeTab="4" xr2:uid="{C63F3EB8-08D2-414D-8217-7DA2F26F8F2E}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="19400" firstSheet="3" activeTab="13" xr2:uid="{C63F3EB8-08D2-414D-8217-7DA2F26F8F2E}"/>
   </bookViews>
   <sheets>
     <sheet name="01 Removing Trend and Season" sheetId="1" r:id="rId1"/>
@@ -26,6 +26,7 @@
     <sheet name="04 Quadratic Trend" sheetId="29" r:id="rId11"/>
     <sheet name="04 Logistic Trend" sheetId="31" r:id="rId12"/>
     <sheet name="04 Summary" sheetId="30" r:id="rId13"/>
+    <sheet name="05 Structural Brakes Analysis" sheetId="32" r:id="rId14"/>
   </sheets>
   <definedNames>
     <definedName name="solver_adj" localSheetId="1" hidden="1">'02 Constant Prices'!$G$38</definedName>
@@ -84,7 +85,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -32191,6 +32192,149 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing8.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>32926</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Picture 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0261B949-0280-1B64-D39A-AEE96301272C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="11589926" cy="8128000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>35626</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>29</xdr:col>
+      <xdr:colOff>807626</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="Picture 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{16468053-0A17-DF53-917F-56C3936B9285}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="13208000" y="35626"/>
+          <a:ext cx="11539126" cy="8092374"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>32</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>35626</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>45</xdr:col>
+      <xdr:colOff>807626</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="Picture 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B9ADAEB2-6321-F043-2EC6-4D5F136E168E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="26416000" y="35626"/>
+          <a:ext cx="11539126" cy="8092374"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -37871,6 +38015,16 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0FBFFF1-1A0E-9D4B-8BE5-1B1C83752C89}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD1526ED-E8A7-8E40-A3AC-3D98D99B61D1}">
   <dimension ref="A1:K43"/>

</xml_diff>